<commit_message>
Update expert review spreadsheet with final discordance resolutions
</commit_message>
<xml_diff>
--- a/Question_Classification/expert_review/discordances_to_review.xlsx
+++ b/Question_Classification/expert_review/discordances_to_review.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filow\OneDrive\Desktop\Repository\ITAMed\Question_Classification\expert_review\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a03553e695d2c46a/Desktop/Repository/ITAMed/Question_Classification/expert_review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF92A03-F12B-40B7-9BA4-C21A3DCC19F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{5EF92A03-F12B-40B7-9BA4-C21A3DCC19F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F9D9F6A-D010-4AFC-A93E-15A85FDD4149}"/>
   <bookViews>
-    <workbookView xWindow="13215" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8670" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Expert Review" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="553">
   <si>
     <t>Anno</t>
   </si>
@@ -2072,8 +2072,8 @@
     <col min="5" max="5" width="40" customWidth="1"/>
     <col min="6" max="7" width="68.3671875" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="40" customWidth="1"/>
-    <col min="10" max="10" width="41.26171875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="0" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7890625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="39.9453125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2130,15 +2130,16 @@
       <c r="G2" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="5"/>
+      <c r="H2" s="5" t="s">
+        <v>128</v>
+      </c>
       <c r="I2" s="5"/>
-      <c r="J2">
+      <c r="J2" t="str">
         <f>IF(I2&lt;&gt;"", H2&amp;"; "&amp;I2,H2)</f>
-        <v>0</v>
-      </c>
-      <c r="K2" t="str">
-        <f>IF(J2&lt;&gt;"", I2&amp;"; "&amp;J2,I2)</f>
-        <v>; 0</v>
+        <v>Anestesia e Rianimazione</v>
+      </c>
+      <c r="K2" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="57.6" x14ac:dyDescent="0.55000000000000004">

</xml_diff>